<commit_message>
Docs: README reescrito a 13 modulos + PROCESO_MENSUAL actualizado + limpieza de basura
- README.md: documentaba 10 modulos desde feb-2026, ahora son 13.
  Sumados BAX-sesiones, Contenidos_mas_disparados y Temas_Consultados.
  D11 pasa de 'otro equipo' a implementado. Link a PROCESO_MENSUAL.md.
- PROCESO_MENSUAL.md: nueva seccion 5.1 (outputs fuera del consolidado),
  9.6 reescrita con el estado real de DescubrirBA-Agente.
- Borrados run_all_old.py y el worktree duplicado .claude/worktrees/.
</commit_message>
<xml_diff>
--- a/No_Entendidos/output/no_entendimiento_agosto_2026.xlsx
+++ b/No_Entendidos/output/no_entendimiento_agosto_2026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.143</v>
+        <v>0.175</v>
       </c>
     </row>
     <row r="14">

</xml_diff>